<commit_message>
Add units to forecast data and refine nav spacing
</commit_message>
<xml_diff>
--- a/data/forecast-all.xlsx
+++ b/data/forecast-all.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="46">
   <si>
     <t>年份</t>
   </si>
@@ -169,6 +169,15 @@
   </si>
   <si>
     <t>预测为“如果……那么……”的条件推演，不是对未来的确定性预测，仅供参考。</t>
+  </si>
+  <si>
+    <t>低预测(万人)</t>
+  </si>
+  <si>
+    <t>中预测(万人)</t>
+  </si>
+  <si>
+    <t>高预测(万人)</t>
   </si>
 </sst>
 </file>
@@ -597,13 +606,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1676,13 +1685,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2755,13 +2764,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -3834,13 +3843,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Unify map source links, fix README copy, and update forecast units
</commit_message>
<xml_diff>
--- a/data/forecast-all.xlsx
+++ b/data/forecast-all.xlsx
@@ -135,7 +135,7 @@
     <t>模型</t>
   </si>
   <si>
-    <t>队列要素法（cohort-component），分性别、单岁年龄，2026—2100 年逐年推演。</t>
+    <t>队列要素法（cohort-component），分性别、单岁年龄，2026~2100 年逐年推演。</t>
   </si>
   <si>
     <t>基准人口</t>
@@ -147,7 +147,7 @@
     <t>历史校准</t>
   </si>
   <si>
-    <t>2021—2025 年出生、死亡、总人口采用国家统计局实际数据；死亡率水平逐年反推匹配实际死亡数。</t>
+    <t>2021~2025 年出生、死亡、总人口采用国家统计局实际数据；死亡率水平逐年反推匹配实际死亡数。</t>
   </si>
   <si>
     <t>生命表/生育率</t>

</xml_diff>